<commit_message>
Update RNR_수입원가_2026_20260909.xlsx 2026-09-09 11:09
</commit_message>
<xml_diff>
--- a/RNR_수입원가_2026_20260909.xlsx
+++ b/RNR_수입원가_2026_20260909.xlsx
@@ -5914,7 +5914,7 @@
         <v>75349820</v>
       </c>
       <c r="L34" s="213" t="n">
-        <v>5186</v>
+        <v>5187</v>
       </c>
       <c r="M34" s="213" t="n">
         <v>3319</v>
@@ -6591,10 +6591,10 @@
         <v>1517.3</v>
       </c>
       <c r="J40" s="128" t="n">
-        <v>74558330</v>
+        <v>74558301</v>
       </c>
       <c r="K40" s="128" t="n">
-        <v>74558330</v>
+        <v>74558301</v>
       </c>
       <c r="L40" s="128" t="n">
         <v>10115</v>
@@ -6706,10 +6706,10 @@
         <v>1517.3</v>
       </c>
       <c r="J41" s="128" t="n">
-        <v>17582284</v>
+        <v>17581259</v>
       </c>
       <c r="K41" s="128" t="n">
-        <v>17582284</v>
+        <v>17581259</v>
       </c>
       <c r="L41" s="128" t="n">
         <v>2385</v>
@@ -7114,7 +7114,7 @@
         </is>
       </c>
       <c r="Y44" s="128" t="n">
-        <v>593662</v>
+        <v>593664</v>
       </c>
       <c r="Z44" s="128">
         <f>S44+W44</f>
@@ -8479,7 +8479,7 @@
         </is>
       </c>
       <c r="Y55" s="128" t="n">
-        <v>45948</v>
+        <v>45946</v>
       </c>
       <c r="Z55" s="128">
         <f>S55+W55</f>
@@ -8626,15 +8626,11 @@
           <t>2025-09</t>
         </is>
       </c>
-      <c r="AE56" s="299" t="inlineStr">
-        <is>
-          <t>2025-09-13</t>
-        </is>
-      </c>
-      <c r="AF56" s="298" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
+      <c r="AE56" s="299" t="n">
+        <v>45913</v>
+      </c>
+      <c r="AF56" s="298" t="n">
+        <v>46262</v>
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
@@ -8751,15 +8747,11 @@
           <t>2025-12</t>
         </is>
       </c>
-      <c r="AE57" s="299" t="inlineStr">
-        <is>
-          <t>2025-12-01</t>
-        </is>
-      </c>
-      <c r="AF57" s="298" t="inlineStr">
-        <is>
-          <t>2026-11-30</t>
-        </is>
+      <c r="AE57" s="299" t="n">
+        <v>45992</v>
+      </c>
+      <c r="AF57" s="298" t="n">
+        <v>46356</v>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
@@ -8876,15 +8868,11 @@
           <t>2025-12</t>
         </is>
       </c>
-      <c r="AE58" s="299" t="inlineStr">
-        <is>
-          <t>2025-12-22</t>
-        </is>
-      </c>
-      <c r="AF58" s="298" t="inlineStr">
-        <is>
-          <t>2026-12-21</t>
-        </is>
+      <c r="AE58" s="299" t="n">
+        <v>46013</v>
+      </c>
+      <c r="AF58" s="298" t="n">
+        <v>46377</v>
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
@@ -9001,15 +8989,11 @@
           <t>2026-01</t>
         </is>
       </c>
-      <c r="AE59" s="299" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="AF59" s="298" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
+      <c r="AE59" s="299" t="n">
+        <v>46023</v>
+      </c>
+      <c r="AF59" s="298" t="n">
+        <v>46387</v>
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1">
@@ -9126,15 +9110,11 @@
           <t>2025-11</t>
         </is>
       </c>
-      <c r="AE60" s="299" t="inlineStr">
-        <is>
-          <t>2025-11-01</t>
-        </is>
-      </c>
-      <c r="AF60" s="298" t="inlineStr">
-        <is>
-          <t>2026-10-30</t>
-        </is>
+      <c r="AE60" s="299" t="n">
+        <v>45962</v>
+      </c>
+      <c r="AF60" s="298" t="n">
+        <v>46325</v>
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1">
@@ -9251,15 +9231,11 @@
           <t>2026-01</t>
         </is>
       </c>
-      <c r="AE61" s="299" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="AF61" s="298" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
+      <c r="AE61" s="299" t="n">
+        <v>46023</v>
+      </c>
+      <c r="AF61" s="298" t="n">
+        <v>46387</v>
       </c>
     </row>
     <row r="62" ht="15.75" customHeight="1">
@@ -9382,15 +9358,11 @@
           <t>2026-01</t>
         </is>
       </c>
-      <c r="AE62" s="299" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="AF62" s="298" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
+      <c r="AE62" s="299" t="n">
+        <v>46023</v>
+      </c>
+      <c r="AF62" s="298" t="n">
+        <v>46387</v>
       </c>
     </row>
     <row r="63" ht="15.75" customHeight="1">
@@ -9507,15 +9479,11 @@
           <t>2026-01</t>
         </is>
       </c>
-      <c r="AE63" s="299" t="inlineStr">
-        <is>
-          <t>2026-01-30</t>
-        </is>
-      </c>
-      <c r="AF63" s="298" t="inlineStr">
-        <is>
-          <t>2027-01-29</t>
-        </is>
+      <c r="AE63" s="299" t="n">
+        <v>46052</v>
+      </c>
+      <c r="AF63" s="298" t="n">
+        <v>46416</v>
       </c>
     </row>
     <row r="64" ht="15.75" customHeight="1">
@@ -9763,15 +9731,11 @@
           <t>2026-01</t>
         </is>
       </c>
-      <c r="AE65" s="299" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="AF65" s="298" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
+      <c r="AE65" s="299" t="n">
+        <v>46023</v>
+      </c>
+      <c r="AF65" s="298" t="n">
+        <v>46387</v>
       </c>
     </row>
     <row r="66" ht="15.75" customHeight="1">
@@ -9888,15 +9852,11 @@
           <t>2026-01</t>
         </is>
       </c>
-      <c r="AE66" s="299" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="AF66" s="298" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
+      <c r="AE66" s="299" t="n">
+        <v>46023</v>
+      </c>
+      <c r="AF66" s="298" t="n">
+        <v>46387</v>
       </c>
     </row>
     <row r="67" ht="15.75" customHeight="1">
@@ -10013,15 +9973,11 @@
           <t>2026-01</t>
         </is>
       </c>
-      <c r="AE67" s="299" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="AF67" s="298" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
+      <c r="AE67" s="299" t="n">
+        <v>46023</v>
+      </c>
+      <c r="AF67" s="298" t="n">
+        <v>46387</v>
       </c>
     </row>
     <row r="68" ht="15.75" customHeight="1">
@@ -10138,15 +10094,11 @@
           <t>2026-03</t>
         </is>
       </c>
-      <c r="AE68" s="299" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
-      </c>
-      <c r="AF68" s="298" t="inlineStr">
-        <is>
-          <t>2027-02-28</t>
-        </is>
+      <c r="AE68" s="299" t="n">
+        <v>46082</v>
+      </c>
+      <c r="AF68" s="298" t="n">
+        <v>46446</v>
       </c>
     </row>
     <row r="69" ht="15.75" customHeight="1">
@@ -10263,15 +10215,11 @@
           <t>2026-01</t>
         </is>
       </c>
-      <c r="AE69" s="299" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="AF69" s="298" t="inlineStr">
-        <is>
-          <t>2027-02-22</t>
-        </is>
+      <c r="AE69" s="299" t="n">
+        <v>46023</v>
+      </c>
+      <c r="AF69" s="298" t="n">
+        <v>46440</v>
       </c>
     </row>
     <row r="70" ht="15.75" customHeight="1">
@@ -10388,15 +10336,11 @@
           <t>2026-03</t>
         </is>
       </c>
-      <c r="AE70" s="299" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
-      </c>
-      <c r="AF70" s="298" t="inlineStr">
-        <is>
-          <t>2027-02-28</t>
-        </is>
+      <c r="AE70" s="299" t="n">
+        <v>46082</v>
+      </c>
+      <c r="AF70" s="298" t="n">
+        <v>46446</v>
       </c>
     </row>
     <row r="71" ht="15.75" customHeight="1">
@@ -10442,10 +10386,10 @@
         <v>753200</v>
       </c>
       <c r="L71" s="302" t="n">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="M71" s="302" t="n">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="N71" s="296" t="inlineStr">
         <is>
@@ -10638,15 +10582,11 @@
           <t>2026-04</t>
         </is>
       </c>
-      <c r="AE72" s="299" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="AF72" s="298" t="inlineStr">
-        <is>
-          <t>2027-03-31</t>
-        </is>
+      <c r="AE72" s="299" t="n">
+        <v>46113</v>
+      </c>
+      <c r="AF72" s="298" t="n">
+        <v>46477</v>
       </c>
     </row>
     <row r="73" ht="15.75" customHeight="1">
@@ -11101,7 +11041,7 @@
       </c>
       <c r="AD76" s="304" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="AE76" s="305" t="n">
@@ -13154,14 +13094,6 @@
     <row r="102">
       <c r="M102" s="40" t="n"/>
     </row>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="A93:G93"/>
@@ -13363,7 +13295,7 @@
         <v>45982</v>
       </c>
       <c r="H4" s="184" t="n">
-        <v>46014</v>
+        <v>46020</v>
       </c>
       <c r="I4" s="184" t="n">
         <v>45992</v>
@@ -14718,43 +14650,6 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
     <row r="70">
       <c r="M70" s="40" t="n"/>
     </row>
@@ -17116,22 +17011,6 @@
         </is>
       </c>
     </row>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
     <row r="71">
       <c r="M71" s="40" t="n"/>
     </row>
@@ -17151,7 +17030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M131"/>
+  <dimension ref="A1:M120"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col width="12.83203125" customWidth="1" style="160" min="1" max="1"/>
@@ -19450,17 +19329,17 @@
           <t>② PO별 비용 안분 내역</t>
         </is>
       </c>
-      <c r="B50" s="333" t="n"/>
-      <c r="C50" s="333" t="n"/>
-      <c r="D50" s="333" t="n"/>
-      <c r="E50" s="333" t="n"/>
-      <c r="F50" s="333" t="n"/>
-      <c r="G50" s="333" t="n"/>
-      <c r="H50" s="333" t="n"/>
-      <c r="I50" s="333" t="n"/>
-      <c r="J50" s="333" t="n"/>
-      <c r="K50" s="333" t="n"/>
-      <c r="L50" s="333" t="n"/>
+      <c r="B50" s="148" t="n"/>
+      <c r="C50" s="148" t="n"/>
+      <c r="D50" s="148" t="n"/>
+      <c r="E50" s="148" t="n"/>
+      <c r="F50" s="148" t="n"/>
+      <c r="G50" s="148" t="n"/>
+      <c r="H50" s="148" t="n"/>
+      <c r="I50" s="148" t="n"/>
+      <c r="J50" s="148" t="n"/>
+      <c r="K50" s="148" t="n"/>
+      <c r="L50" s="149" t="n"/>
       <c r="M50" s="228" t="n"/>
     </row>
     <row r="51" ht="15.75" customHeight="1">
@@ -20831,10 +20710,10 @@
         <v>2299</v>
       </c>
       <c r="J79" s="238" t="n">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="K79" s="238" t="n">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="L79" s="239">
         <f>H79+I79+J79+K79</f>
@@ -21865,7 +21744,7 @@
         <v>12657</v>
       </c>
       <c r="J101" s="238" t="n">
-        <v>5186</v>
+        <v>5187</v>
       </c>
       <c r="K101" s="238" t="n">
         <v>3319</v>
@@ -22000,7 +21879,7 @@
         <v>1517.3</v>
       </c>
       <c r="H104" s="238" t="n">
-        <v>74558330</v>
+        <v>74558301</v>
       </c>
       <c r="I104" s="238" t="n">
         <v>24555</v>
@@ -22047,7 +21926,7 @@
         <v>1517.3</v>
       </c>
       <c r="H105" s="238" t="n">
-        <v>17582284</v>
+        <v>17581259</v>
       </c>
       <c r="I105" s="238" t="n">
         <v>5791</v>
@@ -22761,17 +22640,6 @@
         <v/>
       </c>
     </row>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A50:L50"/>

</xml_diff>